<commit_message>
add "isProjected" and Kickstarter to sales csv export
</commit_message>
<xml_diff>
--- a/docs/backerkit/valid_backerkit.xlsx
+++ b/docs/backerkit/valid_backerkit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelobeng/Documents/ECE_458/hypothetical_publishing/docs/backerkit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600FE0B9-F16D-6C47-9FE1-7008BA5ADCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB39D16C-7AB6-4D4B-804D-714D2F0B4ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="680" windowWidth="28040" windowHeight="16740" xr2:uid="{B8E026E8-973D-C649-9730-50113DE286F7}"/>
+    <workbookView xWindow="380" yWindow="680" windowWidth="12160" windowHeight="16740" xr2:uid="{B8E026E8-973D-C649-9730-50113DE286F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>